<commit_message>
hardware: update device and battery enclosures
</commit_message>
<xml_diff>
--- a/Hardware/BOM/BOM.xlsx
+++ b/Hardware/BOM/BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zoe\Documents\PlatformIO\Projects\CodexLight\Hardware\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FF9BF4D-E3D3-4007-870C-BC0F6891464E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FB3170E-619A-49FC-9643-877B16704C7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -154,7 +154,7 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>MX1.25 Battery-601015</t>
+    <t>MX1.25</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>

</xml_diff>